<commit_message>
Update Functional Testing Report for Cafetron.xlsx
</commit_message>
<xml_diff>
--- a/Deliverables/Functional Testing Report for Cafetron.xlsx
+++ b/Deliverables/Functional Testing Report for Cafetron.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2492171_cognizant_com/Documents/Documents/CAFETRON_TESTING/Deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="13_ncr:1_{93FE7E23-1C99-4CD5-869C-5B188F6F59A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69EBACE1-22B0-4419-BE35-81CB30FB23B9}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="13_ncr:1_{93FE7E23-1C99-4CD5-869C-5B188F6F59A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{981FD8A7-94A1-49DF-8538-D66E298442EA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2288" uniqueCount="1112">
   <si>
     <t>Note</t>
   </si>
@@ -3582,6 +3582,303 @@
   </si>
   <si>
     <t>New</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Password: 12345678; Role: Employee; URL: /login</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Password: 12345678; Role: Vendor; URL: /login</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Password: 12345678; Role: Admin; URL: /login</t>
+  </si>
+  <si>
+    <t>Employee ID: wrong.employee; Password: wrong.password</t>
+  </si>
+  <si>
+    <t>Employee ID: blank; Password: blank</t>
+  </si>
+  <si>
+    <t>Name: QA Employee 20260626; Email: qa_employee_20260626@cafetron.test; Employee ID: QA_EMP_20260626; Password: 12345678; Department: QA Automation; Role: Employee</t>
+  </si>
+  <si>
+    <t>Name: QA Vendor 20260626; Email: qa_vendor_20260626@cafetron.test; Employee ID: QA_VENDOR_20260626; Password: 12345678; Department: QA Automation; Role: Vendor</t>
+  </si>
+  <si>
+    <t>Name: QA Admin 20260626; Email: qa_admin_20260626@cafetron.test; Employee ID: QA_ADMIN_20260626; Password: 12345678; Department: QA Automation; Role: Admin</t>
+  </si>
+  <si>
+    <t>Name: blank; Email: blank; Password: blank; Employee ID: blank; Department: blank</t>
+  </si>
+  <si>
+    <t>Name: QA Invalid Email; Email: invalid-email; Password: 1234567; Employee ID: QA_INVALID_260626; Department: QA</t>
+  </si>
+  <si>
+    <t>Duplicate email: qa_employee_20260626@cafetron.test; Duplicate Employee ID: QA_EMP_20260626; Password: 12345678</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Password: 12345678; Menu date: 2026-06-26; Expected item: QA Test Meal</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Search term: QA Test Meal</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Food type filter: Other; Example item: Vendor item</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Search term: zzzz-no-menu-item</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Item: QA Test Meal; Vendor: QA Vendor 20260626; Quantity: 1; Unit price: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Vendor: QA Vendor 20260626; Quantity: 1; Unit price: Rs 25.00; Expected total: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Quantity: 1; Pickup slot: Evening; Employee ID: QA_EMP_20260626</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Start quantity: 1; Updated quantity: 2; Unit price: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Start quantity: 2; Updated quantity: 1; Unit price: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Start quantity: 1; Action: decrease quantity once</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Quantity: 1; Action: remove item</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Quantity: 1; Action: clear cart</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Checkout date: 2026-06-26; Closed pickup slots: Morning, Afternoon</t>
+  </si>
+  <si>
+    <t>Cart item: QA Test Meal; Pickup slot: Evening or Dinner</t>
+  </si>
+  <si>
+    <t>Item: QA Test Meal; Vendor: QA Vendor 20260626; Quantity: 1; Pickup slot: Evening</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Wallet balance: sufficient; Order total: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Item: QA Test Meal; Quantity: 1; Pickup slot: Evening; Subtotal: Rs 25.00; Wallet balance: sufficient</t>
+  </si>
+  <si>
+    <t>Order ID: 69; Employee ID: QA_EMP_20260626; Expected cart count after order: 0</t>
+  </si>
+  <si>
+    <t>Admin cutoff time: current time minus 1 minute; Employee item: QA Test Meal; Pickup location: QA Cutoff Regression</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Wallet: current employee wallet; Transactions: debit/top-up/refund history</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Order ID: 69; Debit amount: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Order ID: 70; Refund amount: Rs 25.00; Vendor decline reason: Item unavailable</t>
+  </si>
+  <si>
+    <t>Top-up amount: blank; Employee ID: QA_EMP_20260626</t>
+  </si>
+  <si>
+    <t>Top-up amount: -5; Employee ID: QA_EMP_20260626</t>
+  </si>
+  <si>
+    <t>Top-up amount: 10; Expected transaction: TOP_UP Rs 10.00; Employee ID: QA_EMP_20260626</t>
+  </si>
+  <si>
+    <t>Order ID: 69; Item: QA Test Meal; Pickup slot: Evening; Amount: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Order ID: 69; Payment status: PAID; Order status: PENDING_VENDOR; Item: QA Test Meal; Pickup slot: Evening</t>
+  </si>
+  <si>
+    <t>Order ID: 69; Order status: PENDING_VENDOR</t>
+  </si>
+  <si>
+    <t>Order ID: 69; Order status: VENDOR_ACCEPTED; QR route: /pickup/qr/69</t>
+  </si>
+  <si>
+    <t>Order ID: 70; Payment status: REFUNDED; Order status: VENDOR_DECLINED</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Valid QR image for accepted Order ID: 69</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Route: /vendor/scanner</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Browser camera permission state: allowed, blocked, or unavailable</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Assigned Order ID: 69; Item: QA Test Meal; Quantity: 1; Total: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Control data: unrelated order from another vendor</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Pending Order ID: 69; Action: Accept</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Accepted Order ID: 69; Expected status: VENDOR_ACCEPTED</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Pending Order ID: 70; Decline reason: Item unavailable</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Declined Order ID: 70; Expected status: REFUNDED / VENDOR_DECLINED</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Declined Order ID: 70; Expected transaction: REFUND Rs 25.00</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_EMPTY_VENDOR_20260626; Menu state: no items</t>
+  </si>
+  <si>
+    <t>Add Item form data: item name blank; price blank; stock blank; food type blank</t>
+  </si>
+  <si>
+    <t>Item name: QA Test Meal; Price: Rs 25.00; Stock: 5; Food type: Other; Availability: Available</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Search item: QA Test Meal; Vendor: QA Vendor 20260626; Type: Other; Price: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Existing item: QA Test Meal; Updated price: Rs 30.00; Updated stock: 6; Availability: Available</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Dashboard date: 2026-06-26; KPIs: total orders, revenue, items sold, vendor declines</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Dashboard date: 2026-06-26; Range from: 2026-06-26; Range to: 2026-06-26</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Report sections: dashboard summary, daily report, vendor report; Export: CSV / Daily CSV</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Current ordering window: Open; Target state: Closed</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Current ordering window: Closed; Target state: Open</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Cutoff time: current time minus 1 minute; Browser timezone: IST</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Cutoff time input: blank</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor status filter: All; Expected vendor: QA Vendor 20260626</t>
+  </si>
+  <si>
+    <t>Vendor name: QA Admin Vendor 260626; Email: qa.admin.vendor.260626@cafetron.test; Phone: 9876543210; Contact: QA Contact</t>
+  </si>
+  <si>
+    <t>Vendor name: blank; Email: blank; Phone: 9876543210; Contact: QA Contact</t>
+  </si>
+  <si>
+    <t>Logged-out session; Protected routes: /menu, /vendor/orders, /admin, /wallet</t>
+  </si>
+  <si>
+    <t>Logged-out session; Unknown route: /unknown-route-for-test</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor ID: QA_VENDOR_20260626; Direct employee route: /menu</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Restricted routes: /cart, /checkout, /orders, /wallet, /admin</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Routes: /admin, /admin/operations, /admin/vendors, /menu/manage, /pickup/upload, /wallet, /orders, /cart, /checkout</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Name: QA Employee 20260626; Email: qa_employee_20260626@cafetron.test; Department: QA Automation; Role: EMPLOYEE</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Start route: /profile; Action: Logout</t>
+  </si>
+  <si>
+    <t>Accounts: QA_EMP_20260626, QA_VENDOR_20260626, QA_ADMIN_20260626; Verify footer links per role</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Vendor ID: QA_VENDOR_20260626; Item: QA Test Meal; Order ID: 69; Pickup slot: Evening; Wallet balance: sufficient</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Vendor ID: QA_VENDOR_20260626; Item: QA Test Meal; Order ID: 70; Decline reason: Item unavailable; Refund: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Direct route after login: /login</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Direct route after login: /menu</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Start route: /vendor/orders; Control: Back to menu link</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Route: /wallet; Expected control: Logout</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Route: /vendor/queue</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Existing item: QA Test Meal 260626B; Duplicate item name: QA Test Meal 260626B; Price: Rs 25.00; Stock: 5; Type: Other</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Item name: Zero Stock Item 260626; Price: Rs 20.00; Stock: 0; Food type: Snack</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Existing zero-stock item: Zero Stock Item 260626; Stock: 0; Status: UNAVAILABLE</t>
+  </si>
+  <si>
+    <t>Vendor ID: QA_VENDOR_20260626; Existing menu items; Expected locked delete control state</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor dropdown option: QA Admin Vendor 260626; Status options: All, Available, Unavailable</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor filter: QA Vendor 20260626; Expected item: QA Test Meal 260626B</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Existing item: QA Test Meal 260626B; Edit data: unchanged price Rs 25.00, stock 5, type Other</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Dummy item: QA Test Meal 260626B; Price: Rs 12.00; Stock: 0; Action: delete</t>
+  </si>
+  <si>
+    <t>Name: QA Open Admin; Email: qa_open_admin_260626@cafetron.test; Employee ID: QA_OPEN_ADMIN; Password: 12345678; Role: Admin</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Top-up amount: 999999999</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Top-up amount: 10; Browser time: 3:52 PM IST; Displayed wallet time: 10:22 AM</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Employee ID: QA_EMP_20260626; Item: QA Test Meal; Pickup slot: Evening; Order ID: 72; Ordering window: Closed</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Item: QA Test Meal 260626B; Available stock: less than 9; Requested quantity: 9; Unit price: Rs 25.00</t>
+  </si>
+  <si>
+    <t>Employee ID: QA_EMP_20260626; Accepted Order ID: 69; QR route: /pickup/qr/69</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor name: QA Bad Phone; Email: qa.bad.phone.260626@cafetron.test; Phone: ABCphone999999999999999999999999999999; Contact: QA Contact</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Vendor name: QA Bad Phone; Browser time: 3:56 PM IST; Displayed created time: 10:26 AM</t>
+  </si>
+  <si>
+    <t>Admin ID: QA_ADMIN_20260626; Dummy vendor: QA Admin Vendor 260626; Action: delete</t>
   </si>
 </sst>
 </file>
@@ -3696,7 +3993,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -3728,6 +4025,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5160,22 +5460,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="11.453125" customWidth="1"/>
     <col min="3" max="3" width="38.7265625" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="65" customWidth="1"/>
-    <col min="6" max="6" width="58.7265625" customWidth="1"/>
-    <col min="7" max="7" width="18.7265625" customWidth="1"/>
-    <col min="8" max="9" width="11.81640625" customWidth="1"/>
-    <col min="10" max="10" width="16.26953125" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" customWidth="1"/>
+    <col min="5" max="5" width="40" style="12" customWidth="1"/>
+    <col min="6" max="6" width="65" customWidth="1"/>
+    <col min="7" max="7" width="58.7265625" customWidth="1"/>
+    <col min="8" max="8" width="18.7265625" customWidth="1"/>
+    <col min="9" max="10" width="11.81640625" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>47</v>
       </c>
@@ -5189,25 +5490,28 @@
         <v>50</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>1013</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
@@ -5220,26 +5524,29 @@
       <c r="D2" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="13" t="s">
+        <v>1014</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>647</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>648</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="9" t="s">
         <v>649</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="I2" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I2" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J2" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K2" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
@@ -5252,26 +5559,29 @@
       <c r="D3" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="13" t="s">
+        <v>1015</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>650</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>651</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>652</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J3" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>13</v>
       </c>
@@ -5284,26 +5594,29 @@
       <c r="D4" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="13" t="s">
+        <v>1016</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>653</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>654</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>655</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I4" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J4" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>16</v>
       </c>
@@ -5316,26 +5629,29 @@
       <c r="D5" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="13" t="s">
+        <v>1017</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>656</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>657</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>658</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J5" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K5" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>16</v>
       </c>
@@ -5348,26 +5664,29 @@
       <c r="D6" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="13" t="s">
+        <v>1018</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>660</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>661</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>662</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J6" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K6" s="9" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>19</v>
       </c>
@@ -5380,26 +5699,29 @@
       <c r="D7" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="13" t="s">
+        <v>1019</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>664</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>665</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>666</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J7" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K7" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>19</v>
       </c>
@@ -5412,26 +5734,29 @@
       <c r="D8" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="13" t="s">
+        <v>1020</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>668</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>669</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I8" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J8" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K8" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>19</v>
       </c>
@@ -5444,26 +5769,29 @@
       <c r="D9" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="13" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>670</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>671</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>672</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J9" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K9" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>22</v>
       </c>
@@ -5476,26 +5804,29 @@
       <c r="D10" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="13" t="s">
+        <v>1022</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>673</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="H10" s="9" t="s">
         <v>674</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="I10" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J10" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K10" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>22</v>
       </c>
@@ -5508,26 +5839,29 @@
       <c r="D11" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="13" t="s">
+        <v>1023</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>675</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>677</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I11" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J11" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K11" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
@@ -5540,26 +5874,29 @@
       <c r="D12" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="13" t="s">
+        <v>1024</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>678</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>679</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="H12" s="9" t="s">
         <v>680</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I12" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J12" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
@@ -5572,26 +5909,29 @@
       <c r="D13" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="13" t="s">
+        <v>1025</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>681</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>682</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="H13" s="9" t="s">
         <v>879</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="I13" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I13" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J13" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K13" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
@@ -5604,26 +5944,29 @@
       <c r="D14" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="13" t="s">
+        <v>1026</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>880</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>683</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="H14" s="9" t="s">
         <v>881</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="I14" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J14" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K14" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -5636,26 +5979,29 @@
       <c r="D15" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="13" t="s">
+        <v>1027</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>684</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>685</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>882</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I15" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J15" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K15" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -5668,26 +6014,29 @@
       <c r="D16" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="13" t="s">
+        <v>1028</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>686</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>883</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="H16" s="9" t="s">
         <v>884</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="I16" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I16" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J16" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K16" s="9" t="s">
         <v>885</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>28</v>
       </c>
@@ -5700,26 +6049,29 @@
       <c r="D17" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="13" t="s">
+        <v>1029</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>886</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>887</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="I17" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I17" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J17" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K17" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>30</v>
       </c>
@@ -5732,26 +6084,29 @@
       <c r="D18" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="13" t="s">
+        <v>1030</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>689</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="H18" s="9" t="s">
         <v>888</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="I18" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I18" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J18" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K18" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>30</v>
       </c>
@@ -5764,26 +6119,29 @@
       <c r="D19" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="13" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>690</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>889</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="I19" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I19" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J19" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K19" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
@@ -5796,26 +6154,29 @@
       <c r="D20" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="13" t="s">
+        <v>1032</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>691</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>692</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>890</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="I20" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I20" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J20" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K20" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>31</v>
       </c>
@@ -5828,26 +6189,29 @@
       <c r="D21" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="13" t="s">
+        <v>1033</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>693</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>694</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="H21" s="9" t="s">
         <v>891</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="I21" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I21" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J21" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K21" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>31</v>
       </c>
@@ -5860,26 +6224,29 @@
       <c r="D22" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="13" t="s">
+        <v>1034</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>696</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>697</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="H22" s="9" t="s">
         <v>698</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="I22" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I22" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J22" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K22" s="9" t="s">
         <v>892</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>31</v>
       </c>
@@ -5892,26 +6259,29 @@
       <c r="D23" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="13" t="s">
+        <v>1035</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>700</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="H23" s="9" t="s">
         <v>893</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="I23" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I23" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J23" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K23" s="9" t="s">
         <v>894</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
@@ -5924,26 +6294,29 @@
       <c r="D24" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="13" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>701</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>702</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="H24" s="9" t="s">
         <v>703</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="I24" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I24" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J24" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K24" s="9" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>34</v>
       </c>
@@ -5956,26 +6329,29 @@
       <c r="D25" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="13" t="s">
+        <v>1037</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>704</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>705</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="H25" s="9" t="s">
         <v>706</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="I25" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I25" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J25" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K25" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>34</v>
       </c>
@@ -5988,26 +6364,29 @@
       <c r="D26" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="13" t="s">
+        <v>1038</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>707</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>708</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="H26" s="9" t="s">
         <v>709</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="I26" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I26" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J26" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K26" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>34</v>
       </c>
@@ -6020,26 +6399,29 @@
       <c r="D27" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="13" t="s">
+        <v>1039</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>710</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="H27" s="9" t="s">
         <v>895</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="I27" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I27" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J27" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K27" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>34</v>
       </c>
@@ -6052,26 +6434,29 @@
       <c r="D28" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="13" t="s">
+        <v>1040</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>711</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>712</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="H28" s="9" t="s">
         <v>713</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="I28" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I28" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J28" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K28" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>34</v>
       </c>
@@ -6084,26 +6469,29 @@
       <c r="D29" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="13" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>714</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>715</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="H29" s="9" t="s">
         <v>716</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="I29" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I29" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J29" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K29" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>34</v>
       </c>
@@ -6116,26 +6504,29 @@
       <c r="D30" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="13" t="s">
+        <v>1042</v>
+      </c>
+      <c r="F30" s="3" t="s">
         <v>717</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>718</v>
       </c>
-      <c r="G30" s="9" t="s">
+      <c r="H30" s="9" t="s">
         <v>719</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="I30" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I30" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J30" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K30" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>36</v>
       </c>
@@ -6148,26 +6539,29 @@
       <c r="D31" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="13" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>720</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="H31" s="9" t="s">
         <v>896</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="I31" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I31" s="9" t="s">
+      <c r="J31" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="J31" s="9" t="s">
+      <c r="K31" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>37</v>
       </c>
@@ -6180,26 +6574,29 @@
       <c r="D32" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="13" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>721</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="G32" s="3" t="s">
         <v>897</v>
       </c>
-      <c r="G32" s="9" t="s">
+      <c r="H32" s="9" t="s">
         <v>722</v>
       </c>
-      <c r="H32" s="9" t="s">
+      <c r="I32" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I32" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J32" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K32" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>37</v>
       </c>
@@ -6212,26 +6609,29 @@
       <c r="D33" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="13" t="s">
+        <v>1045</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>723</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>724</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="H33" s="9" t="s">
         <v>725</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="I33" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I33" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J33" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K33" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>37</v>
       </c>
@@ -6244,26 +6644,29 @@
       <c r="D34" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="13" t="s">
+        <v>1046</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>726</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>727</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="H34" s="9" t="s">
         <v>728</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="I34" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I34" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J34" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K34" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>40</v>
       </c>
@@ -6276,26 +6679,29 @@
       <c r="D35" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="13" t="s">
+        <v>1047</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>729</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="G35" s="3" t="s">
         <v>730</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="H35" s="9" t="s">
         <v>731</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="I35" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I35" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J35" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K35" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
         <v>40</v>
       </c>
@@ -6308,26 +6714,29 @@
       <c r="D36" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="13" t="s">
+        <v>1048</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>732</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>733</v>
       </c>
-      <c r="G36" s="9" t="s">
+      <c r="H36" s="9" t="s">
         <v>731</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="I36" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I36" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J36" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K36" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>40</v>
       </c>
@@ -6340,26 +6749,29 @@
       <c r="D37" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="13" t="s">
+        <v>1049</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>734</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="G37" s="3" t="s">
         <v>900</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="H37" s="9" t="s">
         <v>735</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="I37" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I37" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J37" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K37" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>43</v>
       </c>
@@ -6372,26 +6784,29 @@
       <c r="D38" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="13" t="s">
+        <v>1050</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="G38" s="3" t="s">
         <v>899</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="H38" s="9" t="s">
         <v>898</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="I38" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I38" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J38" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K38" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>43</v>
       </c>
@@ -6404,26 +6819,29 @@
       <c r="D39" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="13" t="s">
+        <v>1051</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>901</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="G39" s="3" t="s">
         <v>737</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="H39" s="9" t="s">
         <v>738</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="I39" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I39" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J39" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K39" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>45</v>
       </c>
@@ -6436,26 +6854,29 @@
       <c r="D40" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="13" t="s">
+        <v>1052</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>739</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="H40" s="9" t="s">
         <v>740</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="I40" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I40" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J40" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K40" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
         <v>45</v>
       </c>
@@ -6468,26 +6889,29 @@
       <c r="D41" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="13" t="s">
+        <v>1053</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>902</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="G41" s="3" t="s">
         <v>741</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="H41" s="9" t="s">
         <v>742</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="I41" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I41" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J41" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K41" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="s">
         <v>45</v>
       </c>
@@ -6500,26 +6924,29 @@
       <c r="D42" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="13" t="s">
+        <v>1054</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>743</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="G42" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="H42" s="9" t="s">
         <v>744</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="I42" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I42" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J42" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K42" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="116" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" ht="116" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>134</v>
       </c>
@@ -6532,26 +6959,29 @@
       <c r="D43" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="13" t="s">
+        <v>1055</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>922</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="G43" s="3" t="s">
         <v>923</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="H43" s="9" t="s">
         <v>924</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="I43" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I43" s="9" t="s">
+      <c r="J43" s="9" t="s">
         <v>915</v>
       </c>
-      <c r="J43" s="9" t="s">
+      <c r="K43" s="9" t="s">
         <v>925</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>138</v>
       </c>
@@ -6564,26 +6994,29 @@
       <c r="D44" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="13" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>745</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="G44" s="3" t="s">
         <v>746</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="H44" s="9" t="s">
         <v>747</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="I44" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I44" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J44" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K44" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>138</v>
       </c>
@@ -6596,26 +7029,29 @@
       <c r="D45" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="13" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>748</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="G45" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="H45" s="9" t="s">
         <v>749</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="I45" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I45" s="9" t="s">
+      <c r="J45" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="J45" s="9" t="s">
+      <c r="K45" s="9" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>142</v>
       </c>
@@ -6628,26 +7064,29 @@
       <c r="D46" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="13" t="s">
+        <v>1058</v>
+      </c>
+      <c r="F46" s="3" t="s">
         <v>750</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="G46" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="H46" s="9" t="s">
         <v>751</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="I46" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I46" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J46" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K46" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>142</v>
       </c>
@@ -6660,26 +7099,29 @@
       <c r="D47" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="13" t="s">
+        <v>1059</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>752</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="G47" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="H47" s="9" t="s">
         <v>753</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="I47" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I47" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J47" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K47" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>145</v>
       </c>
@@ -6692,26 +7134,29 @@
       <c r="D48" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="13" t="s">
+        <v>1060</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>754</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="3" t="s">
         <v>755</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="H48" s="9" t="s">
         <v>756</v>
       </c>
-      <c r="H48" s="9" t="s">
+      <c r="I48" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I48" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J48" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K48" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
         <v>145</v>
       </c>
@@ -6724,26 +7169,29 @@
       <c r="D49" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E49" s="13" t="s">
+        <v>1061</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>757</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="G49" s="3" t="s">
         <v>758</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>759</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="I49" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I49" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J49" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K49" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
         <v>148</v>
       </c>
@@ -6756,26 +7204,29 @@
       <c r="D50" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="13" t="s">
+        <v>1062</v>
+      </c>
+      <c r="F50" s="3" t="s">
         <v>760</v>
       </c>
-      <c r="F50" s="3" t="s">
+      <c r="G50" s="3" t="s">
         <v>761</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="H50" s="9" t="s">
         <v>762</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="I50" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I50" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J50" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K50" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
         <v>148</v>
       </c>
@@ -6788,26 +7239,29 @@
       <c r="D51" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="E51" s="13" t="s">
+        <v>1063</v>
+      </c>
+      <c r="F51" s="3" t="s">
         <v>763</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="G51" s="3" t="s">
         <v>764</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="H51" s="9" t="s">
         <v>765</v>
       </c>
-      <c r="H51" s="9" t="s">
+      <c r="I51" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I51" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J51" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K51" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
         <v>148</v>
       </c>
@@ -6820,26 +7274,29 @@
       <c r="D52" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="13" t="s">
+        <v>1064</v>
+      </c>
+      <c r="F52" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="F52" s="3" t="s">
+      <c r="G52" s="3" t="s">
         <v>904</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="H52" s="9" t="s">
         <v>905</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="I52" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I52" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J52" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K52" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
         <v>151</v>
       </c>
@@ -6852,26 +7309,29 @@
       <c r="D53" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="E53" s="13" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F53" s="3" t="s">
         <v>767</v>
       </c>
-      <c r="F53" s="3" t="s">
+      <c r="G53" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="H53" s="9" t="s">
         <v>768</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="I53" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I53" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J53" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K53" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
         <v>151</v>
       </c>
@@ -6884,26 +7344,29 @@
       <c r="D54" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="13" t="s">
+        <v>1066</v>
+      </c>
+      <c r="F54" s="3" t="s">
         <v>769</v>
       </c>
-      <c r="F54" s="3" t="s">
+      <c r="G54" s="3" t="s">
         <v>906</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="H54" s="9" t="s">
         <v>907</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="I54" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I54" s="9" t="s">
+      <c r="J54" s="9" t="s">
         <v>908</v>
       </c>
-      <c r="J54" s="9" t="s">
+      <c r="K54" s="9" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="s">
         <v>151</v>
       </c>
@@ -6916,26 +7379,29 @@
       <c r="D55" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E55" s="3" t="s">
+      <c r="E55" s="13" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>770</v>
       </c>
-      <c r="F55" s="3" t="s">
+      <c r="G55" s="3" t="s">
         <v>771</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="H55" s="9" t="s">
         <v>913</v>
       </c>
-      <c r="H55" s="9" t="s">
+      <c r="I55" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I55" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J55" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K55" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="s">
         <v>155</v>
       </c>
@@ -6948,26 +7414,29 @@
       <c r="D56" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="E56" s="13" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F56" s="3" t="s">
         <v>772</v>
       </c>
-      <c r="F56" s="3" t="s">
+      <c r="G56" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="H56" s="9" t="s">
         <v>773</v>
       </c>
-      <c r="H56" s="9" t="s">
+      <c r="I56" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I56" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J56" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K56" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
         <v>155</v>
       </c>
@@ -6980,26 +7449,29 @@
       <c r="D57" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="E57" s="13" t="s">
+        <v>1069</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>774</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="G57" s="3" t="s">
         <v>775</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="H57" s="9" t="s">
         <v>776</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="I57" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I57" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J57" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K57" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="4" t="s">
         <v>158</v>
       </c>
@@ -7012,26 +7484,29 @@
       <c r="D58" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="13" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>777</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="G58" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="H58" s="9" t="s">
         <v>778</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="I58" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I58" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J58" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K58" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="4" t="s">
         <v>161</v>
       </c>
@@ -7044,26 +7519,29 @@
       <c r="D59" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E59" s="13" t="s">
+        <v>1071</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>779</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="G59" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="G59" s="9" t="s">
+      <c r="H59" s="9" t="s">
         <v>780</v>
       </c>
-      <c r="H59" s="9" t="s">
+      <c r="I59" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I59" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J59" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K59" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A60" s="4" t="s">
         <v>161</v>
       </c>
@@ -7076,26 +7554,29 @@
       <c r="D60" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="E60" s="13" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F60" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="F60" s="3" t="s">
+      <c r="G60" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="H60" s="9" t="s">
         <v>926</v>
       </c>
-      <c r="H60" s="9" t="s">
+      <c r="I60" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I60" s="9" t="s">
+      <c r="J60" s="9" t="s">
         <v>914</v>
       </c>
-      <c r="J60" s="9" t="s">
+      <c r="K60" s="9" t="s">
         <v>927</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="4" t="s">
         <v>164</v>
       </c>
@@ -7108,26 +7589,29 @@
       <c r="D61" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="E61" s="3" t="s">
+      <c r="E61" s="13" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>781</v>
       </c>
-      <c r="F61" s="3" t="s">
+      <c r="G61" s="3" t="s">
         <v>782</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="H61" s="9" t="s">
         <v>783</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="I61" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I61" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J61" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K61" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="s">
         <v>164</v>
       </c>
@@ -7140,26 +7624,29 @@
       <c r="D62" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="E62" s="13" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>784</v>
       </c>
-      <c r="F62" s="3" t="s">
+      <c r="G62" s="3" t="s">
         <v>785</v>
       </c>
-      <c r="G62" s="9" t="s">
+      <c r="H62" s="9" t="s">
         <v>786</v>
       </c>
-      <c r="H62" s="9" t="s">
+      <c r="I62" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I62" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J62" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K62" s="9" t="s">
         <v>916</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A63" s="4" t="s">
         <v>167</v>
       </c>
@@ -7172,26 +7659,29 @@
       <c r="D63" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="E63" s="3" t="s">
+      <c r="E63" s="13" t="s">
+        <v>1075</v>
+      </c>
+      <c r="F63" s="3" t="s">
         <v>787</v>
       </c>
-      <c r="F63" s="3" t="s">
+      <c r="G63" s="3" t="s">
         <v>788</v>
       </c>
-      <c r="G63" s="9" t="s">
+      <c r="H63" s="9" t="s">
         <v>789</v>
       </c>
-      <c r="H63" s="9" t="s">
+      <c r="I63" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I63" s="9" t="s">
+      <c r="J63" s="9" t="s">
         <v>928</v>
       </c>
-      <c r="J63" s="9" t="s">
+      <c r="K63" s="9" t="s">
         <v>929</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A64" s="4" t="s">
         <v>167</v>
       </c>
@@ -7204,26 +7694,29 @@
       <c r="D64" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="E64" s="13" t="s">
+        <v>1076</v>
+      </c>
+      <c r="F64" s="3" t="s">
         <v>790</v>
       </c>
-      <c r="F64" s="3" t="s">
+      <c r="G64" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="G64" s="9" t="s">
+      <c r="H64" s="9" t="s">
         <v>930</v>
       </c>
-      <c r="H64" s="9" t="s">
+      <c r="I64" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I64" s="9" t="s">
+      <c r="J64" s="9" t="s">
         <v>931</v>
       </c>
-      <c r="J64" s="9" t="s">
+      <c r="K64" s="9" t="s">
         <v>929</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A65" s="4" t="s">
         <v>170</v>
       </c>
@@ -7236,26 +7729,29 @@
       <c r="D65" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="E65" s="13" t="s">
+        <v>1077</v>
+      </c>
+      <c r="F65" s="3" t="s">
         <v>791</v>
       </c>
-      <c r="F65" s="3" t="s">
+      <c r="G65" s="3" t="s">
         <v>792</v>
       </c>
-      <c r="G65" s="9" t="s">
+      <c r="H65" s="9" t="s">
         <v>793</v>
       </c>
-      <c r="H65" s="9" t="s">
+      <c r="I65" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I65" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J65" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K65" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="s">
         <v>170</v>
       </c>
@@ -7268,26 +7764,29 @@
       <c r="D66" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="E66" s="13" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F66" s="3" t="s">
         <v>794</v>
       </c>
-      <c r="F66" s="3" t="s">
+      <c r="G66" s="3" t="s">
         <v>795</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="H66" s="9" t="s">
         <v>932</v>
       </c>
-      <c r="H66" s="9" t="s">
+      <c r="I66" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I66" s="9" t="s">
+      <c r="J66" s="9" t="s">
         <v>917</v>
       </c>
-      <c r="J66" s="9" t="s">
+      <c r="K66" s="9" t="s">
         <v>933</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A67" s="4" t="s">
         <v>174</v>
       </c>
@@ -7300,26 +7799,29 @@
       <c r="D67" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="E67" s="3" t="s">
+      <c r="E67" s="13" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>796</v>
       </c>
-      <c r="F67" s="3" t="s">
+      <c r="G67" s="3" t="s">
         <v>797</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="H67" s="9" t="s">
         <v>798</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="I67" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I67" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J67" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K67" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A68" s="4" t="s">
         <v>178</v>
       </c>
@@ -7332,26 +7834,29 @@
       <c r="D68" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="E68" s="13" t="s">
+        <v>1080</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>799</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="G68" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="G68" s="9" t="s">
+      <c r="H68" s="9" t="s">
         <v>800</v>
       </c>
-      <c r="H68" s="9" t="s">
+      <c r="I68" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I68" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J68" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K68" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A69" s="4" t="s">
         <v>178</v>
       </c>
@@ -7364,26 +7869,29 @@
       <c r="D69" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="E69" s="3" t="s">
+      <c r="E69" s="13" t="s">
+        <v>1081</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>801</v>
       </c>
-      <c r="F69" s="3" t="s">
+      <c r="G69" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="G69" s="9" t="s">
+      <c r="H69" s="9" t="s">
         <v>802</v>
       </c>
-      <c r="H69" s="9" t="s">
+      <c r="I69" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I69" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J69" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K69" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A70" s="4" t="s">
         <v>182</v>
       </c>
@@ -7396,26 +7904,29 @@
       <c r="D70" s="3" t="s">
         <v>935</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="13" t="s">
+        <v>1082</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>936</v>
       </c>
-      <c r="F70" s="3" t="s">
+      <c r="G70" s="3" t="s">
         <v>937</v>
       </c>
-      <c r="G70" s="9" t="s">
+      <c r="H70" s="9" t="s">
         <v>938</v>
       </c>
-      <c r="H70" s="9" t="s">
+      <c r="I70" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I70" s="9" t="s">
+      <c r="J70" s="9" t="s">
         <v>918</v>
       </c>
-      <c r="J70" s="9" t="s">
+      <c r="K70" s="9" t="s">
         <v>939</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A71" s="4" t="s">
         <v>185</v>
       </c>
@@ -7428,26 +7939,29 @@
       <c r="D71" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E71" s="3" t="s">
+      <c r="E71" s="13" t="s">
+        <v>1083</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>803</v>
       </c>
-      <c r="F71" s="3" t="s">
+      <c r="G71" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="G71" s="9" t="s">
+      <c r="H71" s="9" t="s">
         <v>804</v>
       </c>
-      <c r="H71" s="9" t="s">
+      <c r="I71" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I71" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J71" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K71" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
         <v>186</v>
       </c>
@@ -7460,26 +7974,29 @@
       <c r="D72" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="E72" s="13" t="s">
+        <v>1084</v>
+      </c>
+      <c r="F72" s="3" t="s">
         <v>805</v>
       </c>
-      <c r="F72" s="3" t="s">
+      <c r="G72" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="G72" s="9" t="s">
+      <c r="H72" s="9" t="s">
         <v>806</v>
       </c>
-      <c r="H72" s="9" t="s">
+      <c r="I72" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I72" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J72" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K72" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
         <v>189</v>
       </c>
@@ -7492,26 +8009,29 @@
       <c r="D73" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="E73" s="3" t="s">
+      <c r="E73" s="13" t="s">
+        <v>1085</v>
+      </c>
+      <c r="F73" s="3" t="s">
         <v>807</v>
       </c>
-      <c r="F73" s="3" t="s">
+      <c r="G73" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="H73" s="9" t="s">
         <v>808</v>
       </c>
-      <c r="H73" s="9" t="s">
+      <c r="I73" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I73" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J73" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K73" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
         <v>189</v>
       </c>
@@ -7524,26 +8044,29 @@
       <c r="D74" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="E74" s="3" t="s">
+      <c r="E74" s="13" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F74" s="3" t="s">
         <v>809</v>
       </c>
-      <c r="F74" s="3" t="s">
+      <c r="G74" s="3" t="s">
         <v>810</v>
       </c>
-      <c r="G74" s="9" t="s">
+      <c r="H74" s="9" t="s">
         <v>811</v>
       </c>
-      <c r="H74" s="9" t="s">
+      <c r="I74" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I74" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J74" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K74" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
         <v>192</v>
       </c>
@@ -7556,26 +8079,29 @@
       <c r="D75" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="E75" s="3" t="s">
+      <c r="E75" s="13" t="s">
+        <v>1087</v>
+      </c>
+      <c r="F75" s="3" t="s">
         <v>812</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="G75" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="G75" s="9" t="s">
+      <c r="H75" s="9" t="s">
         <v>813</v>
       </c>
-      <c r="H75" s="9" t="s">
+      <c r="I75" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I75" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J75" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K75" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
         <v>195</v>
       </c>
@@ -7588,26 +8114,29 @@
       <c r="D76" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="E76" s="3" t="s">
+      <c r="E76" s="13" t="s">
+        <v>1088</v>
+      </c>
+      <c r="F76" s="3" t="s">
         <v>814</v>
       </c>
-      <c r="F76" s="3" t="s">
+      <c r="G76" s="3" t="s">
         <v>815</v>
       </c>
-      <c r="G76" s="9" t="s">
+      <c r="H76" s="9" t="s">
         <v>816</v>
       </c>
-      <c r="H76" s="9" t="s">
+      <c r="I76" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I76" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J76" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K76" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
         <v>195</v>
       </c>
@@ -7620,26 +8149,29 @@
       <c r="D77" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="E77" s="3" t="s">
+      <c r="E77" s="13" t="s">
+        <v>1089</v>
+      </c>
+      <c r="F77" s="3" t="s">
         <v>817</v>
       </c>
-      <c r="F77" s="3" t="s">
+      <c r="G77" s="3" t="s">
         <v>818</v>
       </c>
-      <c r="G77" s="9" t="s">
+      <c r="H77" s="9" t="s">
         <v>819</v>
       </c>
-      <c r="H77" s="9" t="s">
+      <c r="I77" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I77" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="J77" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="K77" s="9" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
         <v>199</v>
       </c>
@@ -7652,26 +8184,29 @@
       <c r="D78" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="E78" s="3" t="s">
+      <c r="E78" s="13" t="s">
+        <v>1090</v>
+      </c>
+      <c r="F78" s="3" t="s">
         <v>820</v>
       </c>
-      <c r="F78" s="3" t="s">
+      <c r="G78" s="3" t="s">
         <v>821</v>
       </c>
-      <c r="G78" s="9" t="s">
+      <c r="H78" s="9" t="s">
         <v>822</v>
       </c>
-      <c r="H78" s="9" t="s">
+      <c r="I78" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I78" s="9" t="s">
+      <c r="J78" s="9" t="s">
         <v>447</v>
       </c>
-      <c r="J78" s="9" t="s">
+      <c r="K78" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A79" s="4" t="s">
         <v>202</v>
       </c>
@@ -7684,26 +8219,29 @@
       <c r="D79" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="E79" s="3" t="s">
+      <c r="E79" s="13" t="s">
+        <v>1091</v>
+      </c>
+      <c r="F79" s="3" t="s">
         <v>823</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="G79" s="3" t="s">
         <v>824</v>
       </c>
-      <c r="G79" s="9" t="s">
+      <c r="H79" s="9" t="s">
         <v>825</v>
       </c>
-      <c r="H79" s="9" t="s">
+      <c r="I79" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I79" s="9" t="s">
+      <c r="J79" s="9" t="s">
         <v>453</v>
       </c>
-      <c r="J79" s="9" t="s">
+      <c r="K79" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A80" s="4" t="s">
         <v>202</v>
       </c>
@@ -7716,26 +8254,29 @@
       <c r="D80" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="E80" s="3" t="s">
+      <c r="E80" s="13" t="s">
+        <v>1092</v>
+      </c>
+      <c r="F80" s="3" t="s">
         <v>826</v>
       </c>
-      <c r="F80" s="3" t="s">
+      <c r="G80" s="3" t="s">
         <v>827</v>
       </c>
-      <c r="G80" s="9" t="s">
+      <c r="H80" s="9" t="s">
         <v>828</v>
       </c>
-      <c r="H80" s="9" t="s">
+      <c r="I80" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I80" s="9" t="s">
+      <c r="J80" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="J80" s="9" t="s">
+      <c r="K80" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="4" t="s">
         <v>237</v>
       </c>
@@ -7748,26 +8289,29 @@
       <c r="D81" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="E81" s="3" t="s">
+      <c r="E81" s="13" t="s">
+        <v>1093</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>829</v>
       </c>
-      <c r="F81" s="3" t="s">
+      <c r="G81" s="3" t="s">
         <v>830</v>
       </c>
-      <c r="G81" s="9" t="s">
+      <c r="H81" s="9" t="s">
         <v>831</v>
       </c>
-      <c r="H81" s="9" t="s">
+      <c r="I81" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I81" s="9" t="s">
+      <c r="J81" s="9" t="s">
         <v>459</v>
       </c>
-      <c r="J81" s="9" t="s">
+      <c r="K81" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A82" s="4" t="s">
         <v>208</v>
       </c>
@@ -7780,26 +8324,29 @@
       <c r="D82" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="E82" s="3" t="s">
+      <c r="E82" s="13" t="s">
+        <v>1094</v>
+      </c>
+      <c r="F82" s="3" t="s">
         <v>832</v>
       </c>
-      <c r="F82" s="3" t="s">
+      <c r="G82" s="3" t="s">
         <v>833</v>
       </c>
-      <c r="G82" s="9" t="s">
+      <c r="H82" s="9" t="s">
         <v>834</v>
       </c>
-      <c r="H82" s="9" t="s">
+      <c r="I82" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I82" s="9" t="s">
+      <c r="J82" s="9" t="s">
         <v>462</v>
       </c>
-      <c r="J82" s="9" t="s">
+      <c r="K82" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A83" s="4" t="s">
         <v>205</v>
       </c>
@@ -7812,26 +8359,29 @@
       <c r="D83" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="E83" s="3" t="s">
+      <c r="E83" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="F83" s="3" t="s">
         <v>835</v>
       </c>
-      <c r="F83" s="3" t="s">
+      <c r="G83" s="3" t="s">
         <v>836</v>
       </c>
-      <c r="G83" s="9" t="s">
+      <c r="H83" s="9" t="s">
         <v>837</v>
       </c>
-      <c r="H83" s="9" t="s">
+      <c r="I83" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I83" s="9" t="s">
+      <c r="J83" s="9" t="s">
         <v>466</v>
       </c>
-      <c r="J83" s="9" t="s">
+      <c r="K83" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="s">
         <v>205</v>
       </c>
@@ -7844,26 +8394,29 @@
       <c r="D84" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="E84" s="3" t="s">
+      <c r="E84" s="13" t="s">
+        <v>1096</v>
+      </c>
+      <c r="F84" s="3" t="s">
         <v>838</v>
       </c>
-      <c r="F84" s="3" t="s">
+      <c r="G84" s="3" t="s">
         <v>839</v>
       </c>
-      <c r="G84" s="9" t="s">
+      <c r="H84" s="9" t="s">
         <v>840</v>
       </c>
-      <c r="H84" s="9" t="s">
+      <c r="I84" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I84" s="9" t="s">
+      <c r="J84" s="9" t="s">
         <v>469</v>
       </c>
-      <c r="J84" s="9" t="s">
+      <c r="K84" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A85" s="4" t="s">
         <v>205</v>
       </c>
@@ -7876,26 +8429,29 @@
       <c r="D85" s="3" t="s">
         <v>472</v>
       </c>
-      <c r="E85" s="3" t="s">
+      <c r="E85" s="13" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F85" s="3" t="s">
         <v>841</v>
       </c>
-      <c r="F85" s="3" t="s">
+      <c r="G85" s="3" t="s">
         <v>842</v>
       </c>
-      <c r="G85" s="9" t="s">
+      <c r="H85" s="9" t="s">
         <v>843</v>
       </c>
-      <c r="H85" s="9" t="s">
+      <c r="I85" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I85" s="9" t="s">
+      <c r="J85" s="9" t="s">
         <v>473</v>
       </c>
-      <c r="J85" s="9" t="s">
+      <c r="K85" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A86" s="4" t="s">
         <v>205</v>
       </c>
@@ -7908,26 +8464,29 @@
       <c r="D86" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="E86" s="3" t="s">
+      <c r="E86" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="F86" s="3" t="s">
         <v>844</v>
       </c>
-      <c r="F86" s="3" t="s">
+      <c r="G86" s="3" t="s">
         <v>845</v>
       </c>
-      <c r="G86" s="9" t="s">
+      <c r="H86" s="9" t="s">
         <v>846</v>
       </c>
-      <c r="H86" s="9" t="s">
+      <c r="I86" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I86" s="9" t="s">
+      <c r="J86" s="9" t="s">
         <v>477</v>
       </c>
-      <c r="J86" s="9" t="s">
+      <c r="K86" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="116" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" ht="116" x14ac:dyDescent="0.35">
       <c r="A87" s="4" t="s">
         <v>211</v>
       </c>
@@ -7940,26 +8499,29 @@
       <c r="D87" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E87" s="3" t="s">
+      <c r="E87" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="F87" s="3" t="s">
         <v>847</v>
       </c>
-      <c r="F87" s="3" t="s">
+      <c r="G87" s="3" t="s">
         <v>848</v>
       </c>
-      <c r="G87" s="9" t="s">
+      <c r="H87" s="9" t="s">
         <v>849</v>
       </c>
-      <c r="H87" s="9" t="s">
+      <c r="I87" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I87" s="9" t="s">
+      <c r="J87" s="9" t="s">
         <v>480</v>
       </c>
-      <c r="J87" s="9" t="s">
+      <c r="K87" s="9" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A88" s="4" t="s">
         <v>211</v>
       </c>
@@ -7972,26 +8534,29 @@
       <c r="D88" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="E88" s="3" t="s">
+      <c r="E88" s="13" t="s">
+        <v>1100</v>
+      </c>
+      <c r="F88" s="3" t="s">
         <v>850</v>
       </c>
-      <c r="F88" s="3" t="s">
+      <c r="G88" s="3" t="s">
         <v>851</v>
       </c>
-      <c r="G88" s="9" t="s">
+      <c r="H88" s="9" t="s">
         <v>852</v>
       </c>
-      <c r="H88" s="9" t="s">
+      <c r="I88" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I88" s="9" t="s">
+      <c r="J88" s="9" t="s">
         <v>485</v>
       </c>
-      <c r="J88" s="9" t="s">
+      <c r="K88" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="4" t="s">
         <v>215</v>
       </c>
@@ -8004,26 +8569,29 @@
       <c r="D89" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E89" s="3" t="s">
+      <c r="E89" s="13" t="s">
+        <v>1101</v>
+      </c>
+      <c r="F89" s="3" t="s">
         <v>853</v>
       </c>
-      <c r="F89" s="3" t="s">
+      <c r="G89" s="3" t="s">
         <v>854</v>
       </c>
-      <c r="G89" s="9" t="s">
+      <c r="H89" s="9" t="s">
         <v>855</v>
       </c>
-      <c r="H89" s="9" t="s">
+      <c r="I89" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I89" s="9" t="s">
+      <c r="J89" s="9" t="s">
         <v>488</v>
       </c>
-      <c r="J89" s="9" t="s">
+      <c r="K89" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A90" s="4" t="s">
         <v>215</v>
       </c>
@@ -8036,26 +8604,29 @@
       <c r="D90" s="3" t="s">
         <v>490</v>
       </c>
-      <c r="E90" s="3" t="s">
+      <c r="E90" s="13" t="s">
+        <v>1102</v>
+      </c>
+      <c r="F90" s="3" t="s">
         <v>856</v>
       </c>
-      <c r="F90" s="3" t="s">
+      <c r="G90" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="G90" s="9" t="s">
+      <c r="H90" s="9" t="s">
         <v>940</v>
       </c>
-      <c r="H90" s="9" t="s">
+      <c r="I90" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I90" s="9" t="s">
+      <c r="J90" s="9" t="s">
         <v>919</v>
       </c>
-      <c r="J90" s="9" t="s">
+      <c r="K90" s="9" t="s">
         <v>941</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A91" s="4" t="s">
         <v>218</v>
       </c>
@@ -8068,26 +8639,29 @@
       <c r="D91" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="E91" s="3" t="s">
+      <c r="E91" s="13" t="s">
+        <v>1103</v>
+      </c>
+      <c r="F91" s="3" t="s">
         <v>857</v>
       </c>
-      <c r="F91" s="3" t="s">
+      <c r="G91" s="3" t="s">
         <v>858</v>
       </c>
-      <c r="G91" s="9" t="s">
+      <c r="H91" s="9" t="s">
         <v>859</v>
       </c>
-      <c r="H91" s="9" t="s">
+      <c r="I91" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I91" s="9" t="s">
+      <c r="J91" s="9" t="s">
         <v>494</v>
       </c>
-      <c r="J91" s="9" t="s">
+      <c r="K91" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="4" t="s">
         <v>222</v>
       </c>
@@ -8100,26 +8674,29 @@
       <c r="D92" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E92" s="3" t="s">
+      <c r="E92" s="13" t="s">
+        <v>1104</v>
+      </c>
+      <c r="F92" s="3" t="s">
         <v>860</v>
       </c>
-      <c r="F92" s="3" t="s">
+      <c r="G92" s="3" t="s">
         <v>861</v>
       </c>
-      <c r="G92" s="9" t="s">
+      <c r="H92" s="9" t="s">
         <v>862</v>
       </c>
-      <c r="H92" s="9" t="s">
+      <c r="I92" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I92" s="9" t="s">
+      <c r="J92" s="9" t="s">
         <v>496</v>
       </c>
-      <c r="J92" s="9" t="s">
+      <c r="K92" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="4" t="s">
         <v>222</v>
       </c>
@@ -8132,26 +8709,29 @@
       <c r="D93" s="3" t="s">
         <v>498</v>
       </c>
-      <c r="E93" s="3" t="s">
+      <c r="E93" s="13" t="s">
+        <v>1105</v>
+      </c>
+      <c r="F93" s="3" t="s">
         <v>863</v>
       </c>
-      <c r="F93" s="3" t="s">
+      <c r="G93" s="3" t="s">
         <v>864</v>
       </c>
-      <c r="G93" s="9" t="s">
+      <c r="H93" s="9" t="s">
         <v>865</v>
       </c>
-      <c r="H93" s="9" t="s">
+      <c r="I93" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I93" s="9" t="s">
+      <c r="J93" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="J93" s="9" t="s">
+      <c r="K93" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A94" s="4" t="s">
         <v>225</v>
       </c>
@@ -8164,26 +8744,29 @@
       <c r="D94" s="3" t="s">
         <v>501</v>
       </c>
-      <c r="E94" s="3" t="s">
+      <c r="E94" s="13" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F94" s="3" t="s">
         <v>866</v>
       </c>
-      <c r="F94" s="3" t="s">
+      <c r="G94" s="3" t="s">
         <v>867</v>
       </c>
-      <c r="G94" s="9" t="s">
+      <c r="H94" s="9" t="s">
         <v>868</v>
       </c>
-      <c r="H94" s="9" t="s">
+      <c r="I94" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I94" s="9" t="s">
+      <c r="J94" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="J94" s="9" t="s">
+      <c r="K94" s="9" t="s">
         <v>503</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A95" s="4" t="s">
         <v>228</v>
       </c>
@@ -8196,26 +8779,29 @@
       <c r="D95" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="E95" s="3" t="s">
+      <c r="E95" s="13" t="s">
+        <v>1107</v>
+      </c>
+      <c r="F95" s="3" t="s">
         <v>869</v>
       </c>
-      <c r="F95" s="3" t="s">
+      <c r="G95" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="G95" s="9" t="s">
+      <c r="H95" s="9" t="s">
         <v>870</v>
       </c>
-      <c r="H95" s="9" t="s">
+      <c r="I95" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I95" s="9" t="s">
+      <c r="J95" s="9" t="s">
         <v>507</v>
       </c>
-      <c r="J95" s="9" t="s">
+      <c r="K95" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A96" s="4" t="s">
         <v>231</v>
       </c>
@@ -8228,26 +8814,29 @@
       <c r="D96" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="E96" s="3" t="s">
+      <c r="E96" s="13" t="s">
+        <v>1107</v>
+      </c>
+      <c r="F96" s="3" t="s">
         <v>869</v>
       </c>
-      <c r="F96" s="3" t="s">
+      <c r="G96" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="G96" s="9" t="s">
+      <c r="H96" s="9" t="s">
         <v>870</v>
       </c>
-      <c r="H96" s="9" t="s">
+      <c r="I96" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I96" s="9" t="s">
+      <c r="J96" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="J96" s="9" t="s">
+      <c r="K96" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A97" s="4" t="s">
         <v>231</v>
       </c>
@@ -8260,26 +8849,29 @@
       <c r="D97" s="3" t="s">
         <v>509</v>
       </c>
-      <c r="E97" s="3" t="s">
+      <c r="E97" s="13" t="s">
+        <v>1108</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>871</v>
       </c>
-      <c r="F97" s="3" t="s">
+      <c r="G97" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="G97" s="9" t="s">
+      <c r="H97" s="9" t="s">
         <v>872</v>
       </c>
-      <c r="H97" s="9" t="s">
+      <c r="I97" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I97" s="9" t="s">
+      <c r="J97" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="J97" s="9" t="s">
+      <c r="K97" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A98" s="4" t="s">
         <v>234</v>
       </c>
@@ -8292,26 +8884,29 @@
       <c r="D98" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E98" s="3" t="s">
+      <c r="E98" s="13" t="s">
+        <v>1109</v>
+      </c>
+      <c r="F98" s="3" t="s">
         <v>873</v>
       </c>
-      <c r="F98" s="3" t="s">
+      <c r="G98" s="3" t="s">
         <v>874</v>
       </c>
-      <c r="G98" s="9" t="s">
+      <c r="H98" s="9" t="s">
         <v>875</v>
       </c>
-      <c r="H98" s="9" t="s">
+      <c r="I98" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I98" s="9" t="s">
+      <c r="J98" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="J98" s="9" t="s">
+      <c r="K98" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A99" s="4" t="s">
         <v>234</v>
       </c>
@@ -8324,26 +8919,29 @@
       <c r="D99" s="3" t="s">
         <v>515</v>
       </c>
-      <c r="E99" s="3" t="s">
+      <c r="E99" s="13" t="s">
+        <v>1110</v>
+      </c>
+      <c r="F99" s="3" t="s">
         <v>876</v>
       </c>
-      <c r="F99" s="3" t="s">
+      <c r="G99" s="3" t="s">
         <v>516</v>
       </c>
-      <c r="G99" s="9" t="s">
+      <c r="H99" s="9" t="s">
         <v>877</v>
       </c>
-      <c r="H99" s="9" t="s">
+      <c r="I99" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I99" s="9" t="s">
+      <c r="J99" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="J99" s="9" t="s">
+      <c r="K99" s="9" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" ht="87" x14ac:dyDescent="0.35">
       <c r="A100" s="4" t="s">
         <v>234</v>
       </c>
@@ -8356,22 +8954,25 @@
       <c r="D100" s="3" t="s">
         <v>518</v>
       </c>
-      <c r="E100" s="3" t="s">
+      <c r="E100" s="13" t="s">
+        <v>1111</v>
+      </c>
+      <c r="F100" s="3" t="s">
         <v>878</v>
       </c>
-      <c r="F100" s="3" t="s">
+      <c r="G100" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="G100" s="9" t="s">
+      <c r="H100" s="9" t="s">
         <v>942</v>
       </c>
-      <c r="H100" s="9" t="s">
+      <c r="I100" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I100" s="9" t="s">
+      <c r="J100" s="9" t="s">
         <v>920</v>
       </c>
-      <c r="J100" s="9" t="s">
+      <c r="K100" s="9" t="s">
         <v>943</v>
       </c>
     </row>

</xml_diff>